<commit_message>
Add user manual generation script for Electric Price Update tool
- Implemented a Python script to generate a user manual in Word format (.docx).
- The manual includes sections such as introduction, folder structure, step-by-step usage guide, file format specifications, and troubleshooting.
- Utilizes the `python-docx` library for document creation and formatting.
- Provides a structured layout with headings, tables, and styled text for clarity.
</commit_message>
<xml_diff>
--- a/MONOPUNTO/152 Datos Monopunto COMUNIDAD DE PROPIETARIOS.xlsx
+++ b/MONOPUNTO/152 Datos Monopunto COMUNIDAD DE PROPIETARIOS.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -426,12 +426,12 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
@@ -512,17 +512,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ELEIA</t>
+          <t>PLANEA ENERGIA</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46209</v>
+        <v>46219</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>46568</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46213</v>
+        <v>46220</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -530,22 +530,22 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.2140865731236269</v>
+        <v>0.185108</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1776397511521125</v>
+        <v>0.171766</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1418357068521347</v>
+        <v>0.146114</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1227895988321102</v>
+        <v>0.122322</v>
       </c>
       <c r="J2" t="n">
-        <v>0.105819034243189</v>
+        <v>0.107205</v>
       </c>
       <c r="K2" t="n">
-        <v>0.1262996316783944</v>
+        <v>0.13204</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -562,17 +562,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ELEIA</t>
+          <t>WATIUM</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46209</v>
+        <v>46219</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>46568</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>46213</v>
+        <v>46220</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -580,430 +580,30 @@
         </is>
       </c>
       <c r="F3" t="n">
+        <v>0.142674</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.142674</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.142674</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.142674</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.142674</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.142674</v>
+      </c>
+      <c r="L3" t="n">
         <v>0</v>
       </c>
-      <c r="G3" t="n">
+      <c r="M3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1.827</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1.5</v>
-      </c>
       <c r="N3" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ENERGYA VM</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46210</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>46568</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>0.186692</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.156747</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.130507</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.109694</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.09471400000000001</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.110292</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ENERGYA VM</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>46210</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>46568</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>2</v>
-      </c>
-      <c r="M5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>IBERDROLA</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>46204</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>46568</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>IBERDROLA</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>46204</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>46568</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>10</v>
-      </c>
-      <c r="M7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>46209</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>46568</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>0.215692</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.180789</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.141614</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.118628</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.103902</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.12468</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>46209</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>46568</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>3.73</v>
-      </c>
-      <c r="M9" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>VISALIA</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>46210</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>46568</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>0.20376</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.161756</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.132449</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.107673</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.088375</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.112552</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>AUDAX</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>46212</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>46568</v>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>46213</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>0.1337</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.1337</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.1337</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.1337</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.1337</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.1337</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>